<commit_message>
Publish Tacen_2026_WC PERFECT (rebuild + rank stamp, PADDLETAGGER_CONTRACT)
Whitewater Format A slalom WC; discipline=slalom; start_times=scheduled;
56 official final ranks stamped; files[] xlsx+sha256; generated_at_utc moved.
</commit_message>
<xml_diff>
--- a/events/Tacen_2026_WC/Tacen_2026_WC_start.xlsx
+++ b/events/Tacen_2026_WC/Tacen_2026_WC_start.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Start" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Republish Tacen_2026_WC: Kayak Cross individual (Time Trials) RANK from official classification (92 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/Tacen_2026_WC/Tacen_2026_WC_start.xlsx
+++ b/events/Tacen_2026_WC/Tacen_2026_WC_start.xlsx
@@ -15827,6 +15827,9 @@
       <c r="K260" t="n">
         <v>259</v>
       </c>
+      <c r="M260" t="n">
+        <v>26</v>
+      </c>
       <c r="R260" t="inlineStr">
         <is>
           <t>PLOCHMANN Amelie</t>
@@ -15890,6 +15893,9 @@
       <c r="K261" t="n">
         <v>260</v>
       </c>
+      <c r="M261" t="n">
+        <v>19</v>
+      </c>
       <c r="R261" t="inlineStr">
         <is>
           <t>COCHRANE Georgina</t>
@@ -15953,6 +15959,9 @@
       <c r="K262" t="n">
         <v>261</v>
       </c>
+      <c r="M262" t="n">
+        <v>34</v>
+      </c>
       <c r="R262" t="inlineStr">
         <is>
           <t>TOMISAWA Kurumi</t>
@@ -16016,6 +16025,9 @@
       <c r="K263" t="n">
         <v>262</v>
       </c>
+      <c r="M263" t="n">
+        <v>20</v>
+      </c>
       <c r="R263" t="inlineStr">
         <is>
           <t>XU Linxi</t>
@@ -16079,6 +16091,9 @@
       <c r="K264" t="n">
         <v>263</v>
       </c>
+      <c r="M264" t="n">
+        <v>31</v>
+      </c>
       <c r="R264" t="inlineStr">
         <is>
           <t>PISTONI Lucia</t>
@@ -16142,6 +16157,9 @@
       <c r="K265" t="n">
         <v>264</v>
       </c>
+      <c r="M265" t="n">
+        <v>10</v>
+      </c>
       <c r="R265" t="inlineStr">
         <is>
           <t>BLUME Mina</t>
@@ -16205,6 +16223,9 @@
       <c r="K266" t="n">
         <v>265</v>
       </c>
+      <c r="M266" t="n">
+        <v>32</v>
+      </c>
       <c r="R266" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -16268,6 +16289,9 @@
       <c r="K267" t="n">
         <v>266</v>
       </c>
+      <c r="M267" t="n">
+        <v>16</v>
+      </c>
       <c r="R267" t="inlineStr">
         <is>
           <t>NOVAK Lea</t>
@@ -16331,6 +16355,9 @@
       <c r="K268" t="n">
         <v>267</v>
       </c>
+      <c r="M268" t="n">
+        <v>30</v>
+      </c>
       <c r="R268" t="inlineStr">
         <is>
           <t>DUC Jessica</t>
@@ -16394,6 +16421,9 @@
       <c r="K269" t="n">
         <v>268</v>
       </c>
+      <c r="M269" t="n">
+        <v>15</v>
+      </c>
       <c r="R269" t="inlineStr">
         <is>
           <t>CHLEBOVA Ivana</t>
@@ -16457,6 +16487,9 @@
       <c r="K270" t="n">
         <v>269</v>
       </c>
+      <c r="M270" t="n">
+        <v>33</v>
+      </c>
       <c r="R270" t="inlineStr">
         <is>
           <t>NAGASU Momoka</t>
@@ -16520,6 +16553,9 @@
       <c r="K271" t="n">
         <v>270</v>
       </c>
+      <c r="M271" t="n">
+        <v>29</v>
+      </c>
       <c r="R271" t="inlineStr">
         <is>
           <t>MATTI Svenja</t>
@@ -16583,6 +16619,9 @@
       <c r="K272" t="n">
         <v>271</v>
       </c>
+      <c r="M272" t="n">
+        <v>14</v>
+      </c>
       <c r="R272" t="inlineStr">
         <is>
           <t>DELASSUS Marjorie</t>
@@ -16646,6 +16685,9 @@
       <c r="K273" t="n">
         <v>272</v>
       </c>
+      <c r="M273" t="n">
+        <v>8</v>
+      </c>
       <c r="R273" t="inlineStr">
         <is>
           <t>SORRIBES Laia</t>
@@ -16709,6 +16751,9 @@
       <c r="K274" t="n">
         <v>273</v>
       </c>
+      <c r="M274" t="n">
+        <v>24</v>
+      </c>
       <c r="R274" t="inlineStr">
         <is>
           <t>PIRRO Paulina</t>
@@ -16772,6 +16817,9 @@
       <c r="K275" t="n">
         <v>274</v>
       </c>
+      <c r="M275" t="n">
+        <v>11</v>
+      </c>
       <c r="R275" t="inlineStr">
         <is>
           <t>BRZESKA Dominika</t>
@@ -16835,6 +16883,9 @@
       <c r="K276" t="n">
         <v>275</v>
       </c>
+      <c r="M276" t="n">
+        <v>35</v>
+      </c>
       <c r="R276" t="inlineStr">
         <is>
           <t>ALTMAN Isabella</t>
@@ -16898,6 +16949,9 @@
       <c r="K277" t="n">
         <v>276</v>
       </c>
+      <c r="M277" t="n">
+        <v>13</v>
+      </c>
       <c r="R277" t="inlineStr">
         <is>
           <t>CHEN Lin</t>
@@ -16961,6 +17015,9 @@
       <c r="K278" t="n">
         <v>277</v>
       </c>
+      <c r="M278" t="n">
+        <v>38</v>
+      </c>
       <c r="R278" t="inlineStr">
         <is>
           <t>PINTERIC Naja</t>
@@ -17024,6 +17081,9 @@
       <c r="K279" t="n">
         <v>278</v>
       </c>
+      <c r="M279" t="n">
+        <v>23</v>
+      </c>
       <c r="R279" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -17087,6 +17147,9 @@
       <c r="K280" t="n">
         <v>279</v>
       </c>
+      <c r="M280" t="n">
+        <v>37</v>
+      </c>
       <c r="R280" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -17150,6 +17213,9 @@
       <c r="K281" t="n">
         <v>280</v>
       </c>
+      <c r="M281" t="n">
+        <v>22</v>
+      </c>
       <c r="R281" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -17213,6 +17279,9 @@
       <c r="K282" t="n">
         <v>281</v>
       </c>
+      <c r="M282" t="n">
+        <v>6</v>
+      </c>
       <c r="R282" t="inlineStr">
         <is>
           <t>PANKOVA Zuzana</t>
@@ -17276,6 +17345,9 @@
       <c r="K283" t="n">
         <v>282</v>
       </c>
+      <c r="M283" t="n">
+        <v>12</v>
+      </c>
       <c r="R283" t="inlineStr">
         <is>
           <t>SAMKOVA Olga</t>
@@ -17339,6 +17411,9 @@
       <c r="K284" t="n">
         <v>283</v>
       </c>
+      <c r="M284" t="n">
+        <v>36</v>
+      </c>
       <c r="R284" t="inlineStr">
         <is>
           <t>LI Shiting</t>
@@ -17402,6 +17477,9 @@
       <c r="K285" t="n">
         <v>284</v>
       </c>
+      <c r="M285" t="n">
+        <v>25</v>
+      </c>
       <c r="R285" t="inlineStr">
         <is>
           <t>TEUNISSEN Lena</t>
@@ -17465,6 +17543,9 @@
       <c r="K286" t="n">
         <v>285</v>
       </c>
+      <c r="M286" t="n">
+        <v>21</v>
+      </c>
       <c r="R286" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -17528,6 +17609,9 @@
       <c r="K287" t="n">
         <v>286</v>
       </c>
+      <c r="M287" t="n">
+        <v>18</v>
+      </c>
       <c r="R287" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -17591,6 +17675,9 @@
       <c r="K288" t="n">
         <v>287</v>
       </c>
+      <c r="M288" t="n">
+        <v>17</v>
+      </c>
       <c r="R288" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -17654,6 +17741,9 @@
       <c r="K289" t="n">
         <v>288</v>
       </c>
+      <c r="M289" t="n">
+        <v>4</v>
+      </c>
       <c r="R289" t="inlineStr">
         <is>
           <t>BEKOVA Katerina</t>
@@ -17717,6 +17807,9 @@
       <c r="K290" t="n">
         <v>289</v>
       </c>
+      <c r="M290" t="n">
+        <v>39</v>
+      </c>
       <c r="R290" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -17780,6 +17873,9 @@
       <c r="K291" t="n">
         <v>290</v>
       </c>
+      <c r="M291" t="n">
+        <v>27</v>
+      </c>
       <c r="R291" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -17843,6 +17939,9 @@
       <c r="K292" t="n">
         <v>291</v>
       </c>
+      <c r="M292" t="n">
+        <v>5</v>
+      </c>
       <c r="R292" t="inlineStr">
         <is>
           <t>ZWOLINSKA Klaudia</t>
@@ -17906,6 +18005,9 @@
       <c r="K293" t="n">
         <v>292</v>
       </c>
+      <c r="M293" t="n">
+        <v>28</v>
+      </c>
       <c r="R293" t="inlineStr">
         <is>
           <t>MARX Alena</t>
@@ -17969,6 +18071,9 @@
       <c r="K294" t="n">
         <v>293</v>
       </c>
+      <c r="M294" t="n">
+        <v>7</v>
+      </c>
       <c r="R294" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -18032,6 +18137,9 @@
       <c r="K295" t="n">
         <v>294</v>
       </c>
+      <c r="M295" t="n">
+        <v>9</v>
+      </c>
       <c r="R295" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -18095,6 +18203,9 @@
       <c r="K296" t="n">
         <v>295</v>
       </c>
+      <c r="M296" t="n">
+        <v>3</v>
+      </c>
       <c r="R296" t="inlineStr">
         <is>
           <t>WOODS Kimberley</t>
@@ -18158,6 +18269,9 @@
       <c r="K297" t="n">
         <v>296</v>
       </c>
+      <c r="M297" t="n">
+        <v>1</v>
+      </c>
       <c r="R297" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -18221,6 +18335,9 @@
       <c r="K298" t="n">
         <v>297</v>
       </c>
+      <c r="M298" t="n">
+        <v>2</v>
+      </c>
       <c r="R298" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -18284,6 +18401,9 @@
       <c r="K299" t="n">
         <v>298</v>
       </c>
+      <c r="M299" t="n">
+        <v>35</v>
+      </c>
       <c r="R299" t="inlineStr">
         <is>
           <t>PARRY Daniel</t>
@@ -18347,6 +18467,9 @@
       <c r="K300" t="n">
         <v>299</v>
       </c>
+      <c r="M300" t="n">
+        <v>26</v>
+      </c>
       <c r="R300" t="inlineStr">
         <is>
           <t>BROWN Ben Jacob</t>
@@ -18410,6 +18533,9 @@
       <c r="K301" t="n">
         <v>300</v>
       </c>
+      <c r="M301" t="n">
+        <v>50</v>
+      </c>
       <c r="R301" t="inlineStr">
         <is>
           <t>COWAN Padraig</t>
@@ -18473,6 +18599,9 @@
       <c r="K302" t="n">
         <v>301</v>
       </c>
+      <c r="M302" t="n">
+        <v>43</v>
+      </c>
       <c r="R302" t="inlineStr">
         <is>
           <t>YAMAMOTO Keigo</t>
@@ -18536,6 +18665,9 @@
       <c r="K303" t="n">
         <v>302</v>
       </c>
+      <c r="M303" t="n">
+        <v>48</v>
+      </c>
       <c r="R303" t="inlineStr">
         <is>
           <t>KRAMER Jernej</t>
@@ -18599,6 +18731,9 @@
       <c r="K304" t="n">
         <v>303</v>
       </c>
+      <c r="M304" t="n">
+        <v>40</v>
+      </c>
       <c r="R304" t="inlineStr">
         <is>
           <t>WENG Jize</t>
@@ -18662,6 +18797,9 @@
       <c r="K305" t="n">
         <v>304</v>
       </c>
+      <c r="M305" t="n">
+        <v>42</v>
+      </c>
       <c r="R305" t="inlineStr">
         <is>
           <t>HENDRICK Noel</t>
@@ -18725,6 +18863,9 @@
       <c r="K306" t="n">
         <v>305</v>
       </c>
+      <c r="M306" t="n">
+        <v>45</v>
+      </c>
       <c r="R306" t="inlineStr">
         <is>
           <t>WESTFALL Tyler</t>
@@ -18788,6 +18929,9 @@
       <c r="K307" t="n">
         <v>306</v>
       </c>
+      <c r="M307" t="n">
+        <v>30</v>
+      </c>
       <c r="R307" t="inlineStr">
         <is>
           <t>KONRAD Marten</t>
@@ -18851,6 +18995,9 @@
       <c r="K308" t="n">
         <v>307</v>
       </c>
+      <c r="M308" t="n">
+        <v>12</v>
+      </c>
       <c r="R308" t="inlineStr">
         <is>
           <t>HELLO Joris</t>
@@ -18914,6 +19061,9 @@
       <c r="K309" t="n">
         <v>308</v>
       </c>
+      <c r="M309" t="n">
+        <v>51</v>
+      </c>
       <c r="R309" t="inlineStr">
         <is>
           <t>SEVCIK Matej</t>
@@ -18977,6 +19127,9 @@
       <c r="K310" t="n">
         <v>309</v>
       </c>
+      <c r="M310" t="n">
+        <v>5</v>
+      </c>
       <c r="R310" t="inlineStr">
         <is>
           <t>SMOLEN Michal</t>
@@ -19040,6 +19193,9 @@
       <c r="K311" t="n">
         <v>310</v>
       </c>
+      <c r="M311" t="n">
+        <v>39</v>
+      </c>
       <c r="R311" t="inlineStr">
         <is>
           <t>ROZENTALS Klass Francisks</t>
@@ -19103,6 +19259,9 @@
       <c r="K312" t="n">
         <v>311</v>
       </c>
+      <c r="M312" t="n">
+        <v>47</v>
+      </c>
       <c r="R312" t="inlineStr">
         <is>
           <t>BARAT Andy</t>
@@ -19166,6 +19325,9 @@
       <c r="K313" t="n">
         <v>312</v>
       </c>
+      <c r="M313" t="n">
+        <v>24</v>
+      </c>
       <c r="R313" t="inlineStr">
         <is>
           <t>BARTA Jan</t>
@@ -19229,6 +19391,9 @@
       <c r="K314" t="n">
         <v>313</v>
       </c>
+      <c r="M314" t="n">
+        <v>25</v>
+      </c>
       <c r="R314" t="inlineStr">
         <is>
           <t>UKALOVIC Thomas</t>
@@ -19292,6 +19457,9 @@
       <c r="K315" t="n">
         <v>314</v>
       </c>
+      <c r="M315" t="n">
+        <v>34</v>
+      </c>
       <c r="R315" t="inlineStr">
         <is>
           <t>DIETZ Enrico</t>
@@ -19355,6 +19523,9 @@
       <c r="K316" t="n">
         <v>315</v>
       </c>
+      <c r="M316" t="n">
+        <v>53</v>
+      </c>
       <c r="R316" t="inlineStr">
         <is>
           <t>SOVKO Serhii</t>
@@ -19418,6 +19589,9 @@
       <c r="K317" t="n">
         <v>316</v>
       </c>
+      <c r="M317" t="n">
+        <v>32</v>
+      </c>
       <c r="R317" t="inlineStr">
         <is>
           <t>KRACHKO Arkhyp</t>
@@ -19481,6 +19655,9 @@
       <c r="K318" t="n">
         <v>317</v>
       </c>
+      <c r="M318" t="n">
+        <v>38</v>
+      </c>
       <c r="R318" t="inlineStr">
         <is>
           <t>KOPECEK Michal</t>
@@ -19544,6 +19721,9 @@
       <c r="K319" t="n">
         <v>318</v>
       </c>
+      <c r="M319" t="n">
+        <v>29</v>
+      </c>
       <c r="R319" t="inlineStr">
         <is>
           <t>HAYLETT Ben</t>
@@ -19607,6 +19787,9 @@
       <c r="K320" t="n">
         <v>319</v>
       </c>
+      <c r="M320" t="n">
+        <v>21</v>
+      </c>
       <c r="R320" t="inlineStr">
         <is>
           <t>FEHLMANN Nicolas</t>
@@ -19670,6 +19853,9 @@
       <c r="K321" t="n">
         <v>320</v>
       </c>
+      <c r="M321" t="n">
+        <v>20</v>
+      </c>
       <c r="R321" t="inlineStr">
         <is>
           <t>GALEA Riley</t>
@@ -19733,6 +19919,9 @@
       <c r="K322" t="n">
         <v>321</v>
       </c>
+      <c r="M322" t="n">
+        <v>52</v>
+      </c>
       <c r="R322" t="inlineStr">
         <is>
           <t>KREMSLEHNER Moritz</t>
@@ -19796,6 +19985,9 @@
       <c r="K323" t="n">
         <v>322</v>
       </c>
+      <c r="M323" t="n">
+        <v>15</v>
+      </c>
       <c r="R323" t="inlineStr">
         <is>
           <t>FEDORENKO Oleksandr</t>
@@ -19859,6 +20051,9 @@
       <c r="K324" t="n">
         <v>323</v>
       </c>
+      <c r="M324" t="n">
+        <v>13</v>
+      </c>
       <c r="R324" t="inlineStr">
         <is>
           <t>PISTONI Michele</t>
@@ -19922,6 +20117,9 @@
       <c r="K325" t="n">
         <v>324</v>
       </c>
+      <c r="M325" t="n">
+        <v>36</v>
+      </c>
       <c r="R325" t="inlineStr">
         <is>
           <t>SACHERS Felix</t>
@@ -19985,6 +20183,9 @@
       <c r="K326" t="n">
         <v>325</v>
       </c>
+      <c r="M326" t="n">
+        <v>28</v>
+      </c>
       <c r="R326" t="inlineStr">
         <is>
           <t>PASIUT Michal</t>
@@ -20048,6 +20249,9 @@
       <c r="K327" t="n">
         <v>326</v>
       </c>
+      <c r="M327" t="n">
+        <v>33</v>
+      </c>
       <c r="R327" t="inlineStr">
         <is>
           <t>LEITNER Mario</t>
@@ -20111,6 +20315,9 @@
       <c r="K328" t="n">
         <v>327</v>
       </c>
+      <c r="M328" t="n">
+        <v>46</v>
+      </c>
       <c r="R328" t="inlineStr">
         <is>
           <t>CROSBEE Mark</t>
@@ -20174,6 +20381,9 @@
       <c r="K329" t="n">
         <v>328</v>
       </c>
+      <c r="M329" t="n">
+        <v>37</v>
+      </c>
       <c r="R329" t="inlineStr">
         <is>
           <t>FRIEDENSON Kaelin</t>
@@ -20237,6 +20447,9 @@
       <c r="K330" t="n">
         <v>329</v>
       </c>
+      <c r="M330" t="n">
+        <v>41</v>
+      </c>
       <c r="R330" t="inlineStr">
         <is>
           <t>SAVLI Jakob</t>
@@ -20300,6 +20513,9 @@
       <c r="K331" t="n">
         <v>330</v>
       </c>
+      <c r="M331" t="n">
+        <v>27</v>
+      </c>
       <c r="R331" t="inlineStr">
         <is>
           <t>PUCHNER Oliver</t>
@@ -20363,6 +20579,9 @@
       <c r="K332" t="n">
         <v>331</v>
       </c>
+      <c r="M332" t="n">
+        <v>18</v>
+      </c>
       <c r="R332" t="inlineStr">
         <is>
           <t>ECHANIZ Pau</t>
@@ -20426,6 +20645,9 @@
       <c r="K333" t="n">
         <v>332</v>
       </c>
+      <c r="M333" t="n">
+        <v>49</v>
+      </c>
       <c r="R333" t="inlineStr">
         <is>
           <t>HALCIN Martin</t>
@@ -20489,6 +20711,9 @@
       <c r="K334" t="n">
         <v>333</v>
       </c>
+      <c r="M334" t="n">
+        <v>16</v>
+      </c>
       <c r="R334" t="inlineStr">
         <is>
           <t>FERRAZZI Xabier</t>
@@ -20552,6 +20777,9 @@
       <c r="K335" t="n">
         <v>334</v>
       </c>
+      <c r="M335" t="n">
+        <v>11</v>
+      </c>
       <c r="R335" t="inlineStr">
         <is>
           <t>OSCHMAUTZ Felix</t>
@@ -20615,6 +20843,9 @@
       <c r="K336" t="n">
         <v>335</v>
       </c>
+      <c r="M336" t="n">
+        <v>19</v>
+      </c>
       <c r="R336" t="inlineStr">
         <is>
           <t>CONTRERAS Manel</t>
@@ -20678,6 +20909,9 @@
       <c r="K337" t="n">
         <v>336</v>
       </c>
+      <c r="M337" t="n">
+        <v>44</v>
+      </c>
       <c r="R337" t="inlineStr">
         <is>
           <t>QUAN Xin</t>
@@ -20741,6 +20975,9 @@
       <c r="K338" t="n">
         <v>337</v>
       </c>
+      <c r="M338" t="n">
+        <v>23</v>
+      </c>
       <c r="R338" t="inlineStr">
         <is>
           <t>HU Zhaoshan</t>
@@ -20804,6 +21041,9 @@
       <c r="K339" t="n">
         <v>338</v>
       </c>
+      <c r="M339" t="n">
+        <v>17</v>
+      </c>
       <c r="R339" t="inlineStr">
         <is>
           <t>MARX Dimitri</t>
@@ -20867,6 +21107,9 @@
       <c r="K340" t="n">
         <v>339</v>
       </c>
+      <c r="M340" t="n">
+        <v>8</v>
+      </c>
       <c r="R340" t="inlineStr">
         <is>
           <t>DELFOUR Lucien</t>
@@ -20930,6 +21173,9 @@
       <c r="K341" t="n">
         <v>340</v>
       </c>
+      <c r="M341" t="n">
+        <v>9</v>
+      </c>
       <c r="R341" t="inlineStr">
         <is>
           <t>DE GENNARO Giovanni</t>
@@ -20993,6 +21239,9 @@
       <c r="K342" t="n">
         <v>341</v>
       </c>
+      <c r="M342" t="n">
+        <v>31</v>
+      </c>
       <c r="R342" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -21056,6 +21305,9 @@
       <c r="K343" t="n">
         <v>342</v>
       </c>
+      <c r="M343" t="n">
+        <v>6</v>
+      </c>
       <c r="R343" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -21119,6 +21371,9 @@
       <c r="K344" t="n">
         <v>343</v>
       </c>
+      <c r="M344" t="n">
+        <v>22</v>
+      </c>
       <c r="R344" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -21182,6 +21437,9 @@
       <c r="K345" t="n">
         <v>344</v>
       </c>
+      <c r="M345" t="n">
+        <v>7</v>
+      </c>
       <c r="R345" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -21245,6 +21503,9 @@
       <c r="K346" t="n">
         <v>345</v>
       </c>
+      <c r="M346" t="n">
+        <v>3</v>
+      </c>
       <c r="R346" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -21308,6 +21569,9 @@
       <c r="K347" t="n">
         <v>346</v>
       </c>
+      <c r="M347" t="n">
+        <v>1</v>
+      </c>
       <c r="R347" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -21371,6 +21635,9 @@
       <c r="K348" t="n">
         <v>347</v>
       </c>
+      <c r="M348" t="n">
+        <v>14</v>
+      </c>
       <c r="R348" t="inlineStr">
         <is>
           <t>POLACZYK Mateusz</t>
@@ -21434,6 +21701,9 @@
       <c r="K349" t="n">
         <v>348</v>
       </c>
+      <c r="M349" t="n">
+        <v>2</v>
+      </c>
       <c r="R349" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -21497,6 +21767,9 @@
       <c r="K350" t="n">
         <v>349</v>
       </c>
+      <c r="M350" t="n">
+        <v>10</v>
+      </c>
       <c r="R350" t="inlineStr">
         <is>
           <t>BUTCHER Finn</t>
@@ -21559,6 +21832,9 @@
       </c>
       <c r="K351" t="n">
         <v>350</v>
+      </c>
+      <c r="M351" t="n">
+        <v>4</v>
       </c>
       <c r="R351" t="inlineStr">
         <is>

</xml_diff>